<commit_message>
changing the range style
</commit_message>
<xml_diff>
--- a/тест/template_import.xlsx
+++ b/тест/template_import.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bushk\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\тестовые проекты\ConsoleApp1\тест\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC0335D2-21F4-4D50-B264-91B1444BB30F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{305A880E-238D-4F08-94C8-DAED207DB123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BFB85DB4-43AE-40EF-B987-D893036F1326}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{BFB85DB4-43AE-40EF-B987-D893036F1326}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -119,10 +119,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -447,7 +450,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">

</xml_diff>